<commit_message>
generate log graph for set 1
</commit_message>
<xml_diff>
--- a/compare_results_nodes.xlsx
+++ b/compare_results_nodes.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\ville\OneDrive\Documents\CIC\Tesis\graficas\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6AA2EE6C-6AA9-462B-AD44-8C8EF7630343}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1D96B00E-B1EC-471D-B301-0944BDAF81F3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="14295" yWindow="0" windowWidth="14610" windowHeight="15585" firstSheet="1" activeTab="1" xr2:uid="{D65B6D81-33C6-46CB-ACDB-0F8DE9CD1457}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" firstSheet="1" activeTab="10" xr2:uid="{D65B6D81-33C6-46CB-ACDB-0F8DE9CD1457}"/>
   </bookViews>
   <sheets>
     <sheet name="compare_results_1_nodes" sheetId="1" r:id="rId1"/>
@@ -19,6 +19,11 @@
     <sheet name="compare_times" sheetId="4" r:id="rId4"/>
     <sheet name="compare_solutions" sheetId="5" r:id="rId5"/>
     <sheet name="Sheet1" sheetId="6" r:id="rId6"/>
+    <sheet name="fortimes" sheetId="7" r:id="rId7"/>
+    <sheet name="timegreedy" sheetId="8" r:id="rId8"/>
+    <sheet name="time1" sheetId="9" r:id="rId9"/>
+    <sheet name="time2" sheetId="10" r:id="rId10"/>
+    <sheet name="time3" sheetId="11" r:id="rId11"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -38,7 +43,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="702" uniqueCount="277">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="732" uniqueCount="283">
   <si>
     <t>experiment</t>
   </si>
@@ -869,6 +874,24 @@
   </si>
   <si>
     <t>Rollout k=2</t>
+  </si>
+  <si>
+    <t>20</t>
+  </si>
+  <si>
+    <t>25</t>
+  </si>
+  <si>
+    <t>40</t>
+  </si>
+  <si>
+    <t>50</t>
+  </si>
+  <si>
+    <t>75</t>
+  </si>
+  <si>
+    <t>100</t>
   </si>
 </sst>
 </file>
@@ -1021,7 +1044,7 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="34">
+  <fills count="35">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -1207,8 +1230,14 @@
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="4" tint="0.79998168889431442"/>
+        <bgColor theme="4" tint="0.79998168889431442"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="10">
+  <borders count="14">
     <border>
       <left/>
       <right/>
@@ -1323,6 +1352,50 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="thin">
+        <color theme="4" tint="0.39997558519241921"/>
+      </top>
+      <bottom style="thin">
+        <color theme="4" tint="0.39997558519241921"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color theme="4" tint="0.39997558519241921"/>
+      </right>
+      <top style="thin">
+        <color theme="4" tint="0.39997558519241921"/>
+      </top>
+      <bottom style="thin">
+        <color theme="4" tint="0.39997558519241921"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="thin">
+        <color theme="4" tint="0.39997558519241921"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color theme="4" tint="0.39997558519241921"/>
+      </right>
+      <top style="thin">
+        <color theme="4" tint="0.39997558519241921"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="42">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
@@ -1368,7 +1441,7 @@
     <xf numFmtId="0" fontId="1" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="1" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="7">
+  <cellXfs count="15">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="11" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
@@ -1378,6 +1451,14 @@
     <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="0" fillId="33" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="2" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="0" fontId="0" fillId="34" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="34" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="33" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="33" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="42">
     <cellStyle name="20% - Accent1" xfId="19" builtinId="30" customBuiltin="1"/>
@@ -1423,24 +1504,716 @@
     <cellStyle name="Total" xfId="17" builtinId="25" customBuiltin="1"/>
     <cellStyle name="Warning Text" xfId="14" builtinId="11" customBuiltin="1"/>
   </cellStyles>
-  <dxfs count="24">
+  <dxfs count="52">
     <dxf>
-      <numFmt numFmtId="2" formatCode="0.00"/>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <name val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </font>
     </dxf>
     <dxf>
-      <numFmt numFmtId="2" formatCode="0.00"/>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <name val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </font>
+      <border diagonalUp="0" diagonalDown="0">
+        <left/>
+        <right style="thin">
+          <color theme="4" tint="0.39997558519241921"/>
+        </right>
+        <top style="thin">
+          <color theme="4" tint="0.39997558519241921"/>
+        </top>
+        <bottom style="thin">
+          <color theme="4" tint="0.39997558519241921"/>
+        </bottom>
+        <vertical/>
+        <horizontal/>
+      </border>
     </dxf>
     <dxf>
-      <numFmt numFmtId="2" formatCode="0.00"/>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <name val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </font>
+      <border diagonalUp="0" diagonalDown="0">
+        <left/>
+        <right style="thin">
+          <color theme="4" tint="0.39997558519241921"/>
+        </right>
+        <top style="thin">
+          <color theme="4" tint="0.39997558519241921"/>
+        </top>
+        <bottom style="thin">
+          <color theme="4" tint="0.39997558519241921"/>
+        </bottom>
+        <vertical/>
+        <horizontal/>
+      </border>
     </dxf>
     <dxf>
-      <numFmt numFmtId="2" formatCode="0.00"/>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <name val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </font>
+      <border diagonalUp="0" diagonalDown="0">
+        <left/>
+        <right style="thin">
+          <color theme="4" tint="0.39997558519241921"/>
+        </right>
+        <top style="thin">
+          <color theme="4" tint="0.39997558519241921"/>
+        </top>
+        <bottom style="thin">
+          <color theme="4" tint="0.39997558519241921"/>
+        </bottom>
+        <vertical/>
+        <horizontal/>
+      </border>
     </dxf>
     <dxf>
-      <numFmt numFmtId="0" formatCode="General"/>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <name val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </font>
+      <border diagonalUp="0" diagonalDown="0">
+        <left/>
+        <right style="thin">
+          <color theme="4" tint="0.39997558519241921"/>
+        </right>
+        <top style="thin">
+          <color theme="4" tint="0.39997558519241921"/>
+        </top>
+        <bottom style="thin">
+          <color theme="4" tint="0.39997558519241921"/>
+        </bottom>
+        <vertical/>
+        <horizontal/>
+      </border>
     </dxf>
     <dxf>
-      <numFmt numFmtId="164" formatCode="0.000"/>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <name val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </font>
+      <border diagonalUp="0" diagonalDown="0">
+        <left/>
+        <right style="thin">
+          <color theme="4" tint="0.39997558519241921"/>
+        </right>
+        <top style="thin">
+          <color theme="4" tint="0.39997558519241921"/>
+        </top>
+        <bottom style="thin">
+          <color theme="4" tint="0.39997558519241921"/>
+        </bottom>
+        <vertical/>
+        <horizontal/>
+      </border>
+    </dxf>
+    <dxf>
+      <border outline="0">
+        <bottom style="thin">
+          <color theme="4" tint="0.39997558519241921"/>
+        </bottom>
+      </border>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <name val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <name val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </font>
+      <border diagonalUp="0" diagonalDown="0">
+        <left/>
+        <right/>
+        <top style="thin">
+          <color theme="4" tint="0.39997558519241921"/>
+        </top>
+        <bottom style="thin">
+          <color theme="4" tint="0.39997558519241921"/>
+        </bottom>
+        <vertical/>
+        <horizontal/>
+      </border>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <name val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </font>
+      <border diagonalUp="0" diagonalDown="0">
+        <left/>
+        <right/>
+        <top style="thin">
+          <color theme="4" tint="0.39997558519241921"/>
+        </top>
+        <bottom style="thin">
+          <color theme="4" tint="0.39997558519241921"/>
+        </bottom>
+        <vertical/>
+        <horizontal/>
+      </border>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <name val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </font>
+      <border diagonalUp="0" diagonalDown="0">
+        <left/>
+        <right/>
+        <top style="thin">
+          <color theme="4" tint="0.39997558519241921"/>
+        </top>
+        <bottom style="thin">
+          <color theme="4" tint="0.39997558519241921"/>
+        </bottom>
+        <vertical/>
+        <horizontal/>
+      </border>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <name val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </font>
+      <border diagonalUp="0" diagonalDown="0">
+        <left/>
+        <right/>
+        <top style="thin">
+          <color theme="4" tint="0.39997558519241921"/>
+        </top>
+        <bottom style="thin">
+          <color theme="4" tint="0.39997558519241921"/>
+        </bottom>
+        <vertical/>
+        <horizontal/>
+      </border>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <name val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </font>
+      <border diagonalUp="0" diagonalDown="0">
+        <left/>
+        <right/>
+        <top style="thin">
+          <color theme="4" tint="0.39997558519241921"/>
+        </top>
+        <bottom style="thin">
+          <color theme="4" tint="0.39997558519241921"/>
+        </bottom>
+        <vertical/>
+        <horizontal/>
+      </border>
+    </dxf>
+    <dxf>
+      <border outline="0">
+        <bottom style="thin">
+          <color theme="4" tint="0.39997558519241921"/>
+        </bottom>
+      </border>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <name val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <name val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </font>
+      <border diagonalUp="0" diagonalDown="0">
+        <left/>
+        <right/>
+        <top style="thin">
+          <color theme="4" tint="0.39997558519241921"/>
+        </top>
+        <bottom style="thin">
+          <color theme="4" tint="0.39997558519241921"/>
+        </bottom>
+        <vertical/>
+        <horizontal/>
+      </border>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <name val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </font>
+      <border diagonalUp="0" diagonalDown="0">
+        <left/>
+        <right/>
+        <top style="thin">
+          <color theme="4" tint="0.39997558519241921"/>
+        </top>
+        <bottom style="thin">
+          <color theme="4" tint="0.39997558519241921"/>
+        </bottom>
+        <vertical/>
+        <horizontal/>
+      </border>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <name val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </font>
+      <border diagonalUp="0" diagonalDown="0">
+        <left/>
+        <right/>
+        <top style="thin">
+          <color theme="4" tint="0.39997558519241921"/>
+        </top>
+        <bottom style="thin">
+          <color theme="4" tint="0.39997558519241921"/>
+        </bottom>
+        <vertical/>
+        <horizontal/>
+      </border>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <name val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </font>
+      <border diagonalUp="0" diagonalDown="0">
+        <left/>
+        <right/>
+        <top style="thin">
+          <color theme="4" tint="0.39997558519241921"/>
+        </top>
+        <bottom style="thin">
+          <color theme="4" tint="0.39997558519241921"/>
+        </bottom>
+        <vertical/>
+        <horizontal/>
+      </border>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <name val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </font>
+      <border diagonalUp="0" diagonalDown="0">
+        <left/>
+        <right/>
+        <top style="thin">
+          <color theme="4" tint="0.39997558519241921"/>
+        </top>
+        <bottom style="thin">
+          <color theme="4" tint="0.39997558519241921"/>
+        </bottom>
+        <vertical/>
+        <horizontal/>
+      </border>
+    </dxf>
+    <dxf>
+      <border outline="0">
+        <bottom style="thin">
+          <color theme="4" tint="0.39997558519241921"/>
+        </bottom>
+      </border>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <name val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <name val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </font>
+      <border diagonalUp="0" diagonalDown="0">
+        <left/>
+        <right/>
+        <top style="thin">
+          <color theme="4" tint="0.39997558519241921"/>
+        </top>
+        <bottom style="thin">
+          <color theme="4" tint="0.39997558519241921"/>
+        </bottom>
+        <vertical/>
+        <horizontal/>
+      </border>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <name val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </font>
+      <border diagonalUp="0" diagonalDown="0">
+        <left/>
+        <right/>
+        <top style="thin">
+          <color theme="4" tint="0.39997558519241921"/>
+        </top>
+        <bottom style="thin">
+          <color theme="4" tint="0.39997558519241921"/>
+        </bottom>
+        <vertical/>
+        <horizontal/>
+      </border>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <name val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </font>
+      <border diagonalUp="0" diagonalDown="0">
+        <left/>
+        <right/>
+        <top style="thin">
+          <color theme="4" tint="0.39997558519241921"/>
+        </top>
+        <bottom style="thin">
+          <color theme="4" tint="0.39997558519241921"/>
+        </bottom>
+        <vertical/>
+        <horizontal/>
+      </border>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <name val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </font>
+      <border diagonalUp="0" diagonalDown="0">
+        <left/>
+        <right/>
+        <top style="thin">
+          <color theme="4" tint="0.39997558519241921"/>
+        </top>
+        <bottom style="thin">
+          <color theme="4" tint="0.39997558519241921"/>
+        </bottom>
+        <vertical/>
+        <horizontal/>
+      </border>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <name val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </font>
+      <border diagonalUp="0" diagonalDown="0">
+        <left/>
+        <right/>
+        <top style="thin">
+          <color theme="4" tint="0.39997558519241921"/>
+        </top>
+        <bottom style="thin">
+          <color theme="4" tint="0.39997558519241921"/>
+        </bottom>
+        <vertical/>
+        <horizontal/>
+      </border>
+    </dxf>
+    <dxf>
+      <border outline="0">
+        <bottom style="thin">
+          <color theme="4" tint="0.39997558519241921"/>
+        </bottom>
+      </border>
     </dxf>
     <dxf>
       <numFmt numFmtId="165" formatCode="0.0000"/>
@@ -1467,6 +2240,18 @@
       <numFmt numFmtId="165" formatCode="0.0000"/>
     </dxf>
     <dxf>
+      <numFmt numFmtId="2" formatCode="0.00"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="2" formatCode="0.00"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="2" formatCode="0.00"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="2" formatCode="0.00"/>
+    </dxf>
+    <dxf>
       <numFmt numFmtId="0" formatCode="General"/>
     </dxf>
     <dxf>
@@ -1474,6 +2259,12 @@
     </dxf>
     <dxf>
       <numFmt numFmtId="0" formatCode="General"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="0" formatCode="General"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="164" formatCode="0.000"/>
     </dxf>
     <dxf>
       <numFmt numFmtId="164" formatCode="0.000"/>
@@ -1553,6 +2344,36 @@
 </table>
 </file>
 
+<file path=xl/tables/table10.xml><?xml version="1.0" encoding="utf-8"?>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="10" xr:uid="{7419CC4E-D46E-4EE6-A21C-75DB50692B20}" name="Table10" displayName="Table10" ref="A1:F11" totalsRowShown="0" dataDxfId="7" tableBorderDxfId="13">
+  <autoFilter ref="A1:F11" xr:uid="{7419CC4E-D46E-4EE6-A21C-75DB50692B20}"/>
+  <tableColumns count="6">
+    <tableColumn id="1" xr3:uid="{C12616F2-F9EF-44FD-B101-59EEED24BA8B}" name="20"/>
+    <tableColumn id="2" xr3:uid="{590898BA-7D25-4912-9C6F-CFD635325FF6}" name="25" dataDxfId="12"/>
+    <tableColumn id="3" xr3:uid="{54CF1FB8-E916-4280-9BA8-E2CF6EC81817}" name="40" dataDxfId="11"/>
+    <tableColumn id="4" xr3:uid="{A19A8795-4407-46E9-B829-B147FCE47CE1}" name="50" dataDxfId="10"/>
+    <tableColumn id="5" xr3:uid="{2C862B69-AE54-4C0B-9BE8-3047BABA19F7}" name="75" dataDxfId="9"/>
+    <tableColumn id="6" xr3:uid="{46534EE3-1978-43ED-82A2-43E67CD3480F}" name="100" dataDxfId="8"/>
+  </tableColumns>
+  <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
+</table>
+</file>
+
+<file path=xl/tables/table11.xml><?xml version="1.0" encoding="utf-8"?>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="11" xr:uid="{A9E9CCCF-D0E5-4746-A6D9-601FFC30B8CE}" name="Table11" displayName="Table11" ref="A1:F11" totalsRowShown="0" dataDxfId="0" tableBorderDxfId="6">
+  <autoFilter ref="A1:F11" xr:uid="{A9E9CCCF-D0E5-4746-A6D9-601FFC30B8CE}"/>
+  <tableColumns count="6">
+    <tableColumn id="1" xr3:uid="{48DDA3A9-0BCE-445A-A853-17FF6476586B}" name="20"/>
+    <tableColumn id="2" xr3:uid="{1EC3B596-9909-4332-9150-FE4A22790396}" name="25" dataDxfId="5"/>
+    <tableColumn id="3" xr3:uid="{3E3FF7E6-502B-428D-8537-291D461FF375}" name="40" dataDxfId="4"/>
+    <tableColumn id="4" xr3:uid="{7433F480-8EFD-4531-9980-1204EEF2A621}" name="50" dataDxfId="3"/>
+    <tableColumn id="5" xr3:uid="{1A2A9B71-7435-437C-9CA7-A315DA80A1DC}" name="75" dataDxfId="2"/>
+    <tableColumn id="6" xr3:uid="{C4B469EF-FA42-4766-8838-AAAC1AABC62D}" name="100" dataDxfId="1"/>
+  </tableColumns>
+  <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
+</table>
+</file>
+
 <file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{162C42B6-0730-401F-B565-376E56EC1620}" name="Table1" displayName="Table1" ref="A1:J7" totalsRowShown="0">
   <autoFilter ref="A1:J7" xr:uid="{162C42B6-0730-401F-B565-376E56EC1620}"/>
@@ -1561,28 +2382,28 @@
     <tableColumn id="2" xr3:uid="{F36D6776-FA9A-482A-9103-7245C0E79EE8}" name="Instancias">
       <calculatedColumnFormula>COUNTIF(compare_results_1_nodes!B:B,comparaciones!A2)</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="3" xr3:uid="{DAAEB182-0D3C-45B3-BEBF-95F9F9EE4E4E}" name="Prom. Nodos salvados óptimo IQCP" dataDxfId="23">
+    <tableColumn id="3" xr3:uid="{DAAEB182-0D3C-45B3-BEBF-95F9F9EE4E4E}" name="Prom. Nodos salvados óptimo IQCP" dataDxfId="51">
       <calculatedColumnFormula>AVERAGEIF(Table2[n_nodes],Table1[[#This Row],[Nodos]],Table2[optimal_iqcp])</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="4" xr3:uid="{ACDA9EFF-3B26-4747-9816-E11EAB637C22}" name="Prom. Nodos salvados Rollout k=1" dataDxfId="22">
+    <tableColumn id="4" xr3:uid="{ACDA9EFF-3B26-4747-9816-E11EAB637C22}" name="Prom. Nodos salvados Rollout k=1" dataDxfId="50">
       <calculatedColumnFormula>AVERAGEIF(Table2[n_nodes],Table1[[#This Row],[Nodos]],Table2[optimal_rollout k=1])</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="5" xr3:uid="{98D79523-EFF5-4762-AAEA-6FEBCD801462}" name="Prom. Nodos salvados Rollout k=2" dataDxfId="21">
+    <tableColumn id="5" xr3:uid="{98D79523-EFF5-4762-AAEA-6FEBCD801462}" name="Prom. Nodos salvados Rollout k=2" dataDxfId="49">
       <calculatedColumnFormula>AVERAGEIF(Table2[n_nodes],Table1[[#This Row],[Nodos]],Table2[optimal_rollout k=2])</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="6" xr3:uid="{EF4A4DDD-CBFD-4414-A3B3-9AABCC93DDE6}" name="Prom. Nodos salvados Rollout k=3" dataDxfId="20">
+    <tableColumn id="6" xr3:uid="{EF4A4DDD-CBFD-4414-A3B3-9AABCC93DDE6}" name="Prom. Nodos salvados Rollout k=3" dataDxfId="48">
       <calculatedColumnFormula>AVERAGEIF(Table2[n_nodes],Table1[[#This Row],[Nodos]],Table2[optimal_rollout k=3])</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="7" xr3:uid="{C5442743-9291-4BEA-8DDB-8BEA32CEA7D0}" name="GAP Rollout k=1" dataDxfId="5">
+    <tableColumn id="7" xr3:uid="{C5442743-9291-4BEA-8DDB-8BEA32CEA7D0}" name="GAP Rollout k=1" dataDxfId="47">
       <calculatedColumnFormula>((Table1[[#This Row],[Prom. Nodos salvados óptimo IQCP]]-Table1[[#This Row],[Prom. Nodos salvados Rollout k=1]])/Table1[[#This Row],[Prom. Nodos salvados óptimo IQCP]])*100</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="8" xr3:uid="{F65166D3-BF5F-4B0B-9BA0-0F2A9C0FFB43}" name="GAP Rollout k=2" dataDxfId="19">
+    <tableColumn id="8" xr3:uid="{F65166D3-BF5F-4B0B-9BA0-0F2A9C0FFB43}" name="GAP Rollout k=2" dataDxfId="46">
       <calculatedColumnFormula>((Table1[[#This Row],[Prom. Nodos salvados óptimo IQCP]]-Table1[[#This Row],[Prom. Nodos salvados Rollout k=2]])/Table1[[#This Row],[Prom. Nodos salvados óptimo IQCP]])*100</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="9" xr3:uid="{F8DBFB38-4A80-4A39-9E67-37DC9A309E50}" name="GAP Rollout k=3" dataDxfId="18">
+    <tableColumn id="9" xr3:uid="{F8DBFB38-4A80-4A39-9E67-37DC9A309E50}" name="GAP Rollout k=3" dataDxfId="45">
       <calculatedColumnFormula>((Table1[[#This Row],[Prom. Nodos salvados óptimo IQCP]]-Table1[[#This Row],[Prom. Nodos salvados Rollout k=3]])/Table1[[#This Row],[Prom. Nodos salvados óptimo IQCP]])*100</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="10" xr3:uid="{4B9484E7-CE8D-4A10-985B-E3F90E5B79B8}" name="Greedy" dataDxfId="17">
+    <tableColumn id="10" xr3:uid="{4B9484E7-CE8D-4A10-985B-E3F90E5B79B8}" name="Greedy" dataDxfId="44">
       <calculatedColumnFormula>AVERAGEIF(Table2[n_nodes],Table1[[#This Row],[Nodos]],Table2[optimal_greedy])</calculatedColumnFormula>
     </tableColumn>
   </tableColumns>
@@ -1595,28 +2416,28 @@
   <autoFilter ref="A12:I18" xr:uid="{65F5BAA4-39EF-45E9-972D-524975488572}"/>
   <tableColumns count="9">
     <tableColumn id="1" xr3:uid="{C609702D-4566-4051-84BD-DD262F5DB361}" name="Nodos"/>
-    <tableColumn id="2" xr3:uid="{D0690FC9-4208-48E7-B589-0202D203BD4C}" name="Instancias" dataDxfId="16">
+    <tableColumn id="2" xr3:uid="{D0690FC9-4208-48E7-B589-0202D203BD4C}" name="Instancias" dataDxfId="43">
       <calculatedColumnFormula>COUNTIF(Table2[n_nodes],Table3[[#This Row],[Nodos]])</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="3" xr3:uid="{7015213A-275D-4E0D-9A3B-65299EF55E20}" name="Prom. T-CPU MIQCP" dataDxfId="15">
+    <tableColumn id="3" xr3:uid="{7015213A-275D-4E0D-9A3B-65299EF55E20}" name="Prom. T-CPU MIQCP" dataDxfId="42">
       <calculatedColumnFormula>AVERAGEIF(Table2[n_nodes],Table3[[#This Row],[Nodos]],Table2[duration_miqcp])</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="4" xr3:uid="{7C651E0C-AF63-467E-86ED-2FD9B5F0E894}" name="Prom. T-CPU IQCP" dataDxfId="14">
+    <tableColumn id="4" xr3:uid="{7C651E0C-AF63-467E-86ED-2FD9B5F0E894}" name="Prom. T-CPU IQCP" dataDxfId="41">
       <calculatedColumnFormula>AVERAGEIF(Table2[n_nodes],Table3[[#This Row],[Nodos]],Table2[duration_iqcp])</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="5" xr3:uid="{4D7253B2-856C-4124-9351-A637A52BE61A}" name="Prom. T-CPU ILP" dataDxfId="4">
+    <tableColumn id="5" xr3:uid="{4D7253B2-856C-4124-9351-A637A52BE61A}" name="Prom. T-CPU ILP" dataDxfId="40">
       <calculatedColumnFormula>AVERAGEIF(Table2[n_nodes],Table3[[#This Row],[Nodos]],Table2[duration_ilp])</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="6" xr3:uid="{DD701191-F57D-495C-96C3-33D794A6591D}" name="Prom. T-CPU Rollout k=1" dataDxfId="3">
+    <tableColumn id="6" xr3:uid="{DD701191-F57D-495C-96C3-33D794A6591D}" name="Prom. T-CPU Rollout k=1" dataDxfId="39">
       <calculatedColumnFormula>AVERAGEIF(Table2[n_nodes],Table3[[#This Row],[Nodos]],Table2[time_taken k=1])</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="7" xr3:uid="{DFE8E634-44A4-4852-8C0D-F1BA07BF8507}" name="Prom. T-CPU Rollout k=2" dataDxfId="2">
+    <tableColumn id="7" xr3:uid="{DFE8E634-44A4-4852-8C0D-F1BA07BF8507}" name="Prom. T-CPU Rollout k=2" dataDxfId="38">
       <calculatedColumnFormula>AVERAGEIF(Table2[n_nodes],Table3[[#This Row],[Nodos]],Table2[time_taken k=2])</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="8" xr3:uid="{10B7E6E4-7C9B-4735-867F-BBE3CC112EA8}" name="Prom. T-CPU Rollout k=3" dataDxfId="1">
+    <tableColumn id="8" xr3:uid="{10B7E6E4-7C9B-4735-867F-BBE3CC112EA8}" name="Prom. T-CPU Rollout k=3" dataDxfId="37">
       <calculatedColumnFormula>AVERAGEIF(Table2[n_nodes],Table3[[#This Row],[Nodos]],Table2[time_taken k=3])</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="9" xr3:uid="{0FA07F6D-7F27-4D79-B873-ECC1770BC9E4}" name="Prom. T-CPU Greedy" dataDxfId="0">
+    <tableColumn id="9" xr3:uid="{0FA07F6D-7F27-4D79-B873-ECC1770BC9E4}" name="Prom. T-CPU Greedy" dataDxfId="36">
       <calculatedColumnFormula>AVERAGEIF(Table2[n_nodes],Table3[[#This Row],[Nodos]],Table2[duration_greedy])</calculatedColumnFormula>
     </tableColumn>
   </tableColumns>
@@ -1649,14 +2470,14 @@
   <tableColumns count="10">
     <tableColumn id="1" xr3:uid="{46A0C2C8-56E5-4A57-8BFD-A60ED7C7916F}" name="id"/>
     <tableColumn id="2" xr3:uid="{667A574A-3BDB-421C-91AF-72CEEB2739F2}" name="n_nodes"/>
-    <tableColumn id="3" xr3:uid="{F1467B7B-2F5E-4DF5-9364-BDE3F3C9E596}" name="duration_dp" dataDxfId="13"/>
-    <tableColumn id="6" xr3:uid="{82CDB484-1F3C-46A0-9206-C53BFA0B71BB}" name="duration_iqcp" dataDxfId="12"/>
-    <tableColumn id="9" xr3:uid="{9BC1E1A5-23F7-4E70-A254-C811A7B0E9AA}" name="duration_ilp" dataDxfId="11"/>
-    <tableColumn id="12" xr3:uid="{CC8D3D03-6199-450C-9270-FA818B49B6F5}" name="duration_miqcp" dataDxfId="10"/>
-    <tableColumn id="15" xr3:uid="{00244C2A-4D1B-43B6-80A6-9F0655A1C8AE}" name="duration_greedy" dataDxfId="9"/>
-    <tableColumn id="19" xr3:uid="{F2D3393D-9B19-43A7-8700-D4DF4F789BAB}" name="duration_rollout k=1" dataDxfId="8"/>
-    <tableColumn id="24" xr3:uid="{1F870097-64C2-4D53-91EE-C831CE7BAE8E}" name="duration_rollout k=2" dataDxfId="7"/>
-    <tableColumn id="29" xr3:uid="{479012F8-DDF3-4D04-847B-5CA8E72CA78B}" name="duration_rollout k=3" dataDxfId="6"/>
+    <tableColumn id="3" xr3:uid="{F1467B7B-2F5E-4DF5-9364-BDE3F3C9E596}" name="duration_dp" dataDxfId="35"/>
+    <tableColumn id="6" xr3:uid="{82CDB484-1F3C-46A0-9206-C53BFA0B71BB}" name="duration_iqcp" dataDxfId="34"/>
+    <tableColumn id="9" xr3:uid="{9BC1E1A5-23F7-4E70-A254-C811A7B0E9AA}" name="duration_ilp" dataDxfId="33"/>
+    <tableColumn id="12" xr3:uid="{CC8D3D03-6199-450C-9270-FA818B49B6F5}" name="duration_miqcp" dataDxfId="32"/>
+    <tableColumn id="15" xr3:uid="{00244C2A-4D1B-43B6-80A6-9F0655A1C8AE}" name="duration_greedy" dataDxfId="31"/>
+    <tableColumn id="19" xr3:uid="{F2D3393D-9B19-43A7-8700-D4DF4F789BAB}" name="duration_rollout k=1" dataDxfId="30"/>
+    <tableColumn id="24" xr3:uid="{1F870097-64C2-4D53-91EE-C831CE7BAE8E}" name="duration_rollout k=2" dataDxfId="29"/>
+    <tableColumn id="29" xr3:uid="{479012F8-DDF3-4D04-847B-5CA8E72CA78B}" name="duration_rollout k=3" dataDxfId="28"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -1671,6 +2492,54 @@
     <tableColumn id="18" xr3:uid="{31EB5B50-BE92-48A0-878C-3271CE2B3AA9}" name="solution_rollout k=1"/>
     <tableColumn id="23" xr3:uid="{5978E5CE-1F36-43B4-B7A6-DBC0A5B31F64}" name="solution_rollout k=2"/>
     <tableColumn id="28" xr3:uid="{56AB7540-FE9A-4D8D-A7F9-5916A5B2F4F1}" name="solution_rollout k=3"/>
+  </tableColumns>
+  <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
+</table>
+</file>
+
+<file path=xl/tables/table7.xml><?xml version="1.0" encoding="utf-8"?>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="7" xr:uid="{DCFBD6C3-3D0C-4AC8-AFA9-DE55E7E26EAC}" name="Table28" displayName="Table28" ref="A1:F61" totalsRowShown="0">
+  <autoFilter ref="A1:F61" xr:uid="{DCFBD6C3-3D0C-4AC8-AFA9-DE55E7E26EAC}"/>
+  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:F61">
+    <sortCondition ref="B1:B61"/>
+  </sortState>
+  <tableColumns count="6">
+    <tableColumn id="1" xr3:uid="{97DDD60E-682D-40F3-BA07-1BA1BFB5C514}" name="experiment"/>
+    <tableColumn id="2" xr3:uid="{6CB3EFF9-AEAF-4166-A292-74F3B4B5B891}" name="n_nodes"/>
+    <tableColumn id="15" xr3:uid="{7C1AC257-35AB-49BB-A41B-DC37F9127EBB}" name="duration_greedy"/>
+    <tableColumn id="19" xr3:uid="{E6EBFC4D-F08F-4839-B0F3-47C80D57EE26}" name="time_taken k=1"/>
+    <tableColumn id="24" xr3:uid="{F88826EC-676C-4FD4-A052-B11D2552F419}" name="time_taken k=2"/>
+    <tableColumn id="29" xr3:uid="{A09D4FA3-DA10-4F27-9CF3-E28D70DB38DF}" name="time_taken k=3"/>
+  </tableColumns>
+  <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
+</table>
+</file>
+
+<file path=xl/tables/table8.xml><?xml version="1.0" encoding="utf-8"?>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="8" xr:uid="{EAC25E40-4EA8-4CBD-AC8B-5B99CF5BA047}" name="Table8" displayName="Table8" ref="A1:F11" totalsRowShown="0" dataDxfId="21" tableBorderDxfId="27">
+  <autoFilter ref="A1:F11" xr:uid="{EAC25E40-4EA8-4CBD-AC8B-5B99CF5BA047}"/>
+  <tableColumns count="6">
+    <tableColumn id="1" xr3:uid="{90AA1423-79D0-47FA-80E4-0F13D63849A9}" name="20"/>
+    <tableColumn id="2" xr3:uid="{A8479BF4-95F6-460A-A7DC-1AAD8174C7CE}" name="25" dataDxfId="26"/>
+    <tableColumn id="3" xr3:uid="{D3EA3B60-C263-4948-8059-906FC1E0687E}" name="40" dataDxfId="25"/>
+    <tableColumn id="4" xr3:uid="{8443D5FB-84DF-4F0F-96CB-F80BA9F06978}" name="50" dataDxfId="24"/>
+    <tableColumn id="5" xr3:uid="{2455CE84-9653-4A99-9A59-87C669730F46}" name="75" dataDxfId="23"/>
+    <tableColumn id="6" xr3:uid="{1AC13411-CC3E-4E04-8981-8ED887637298}" name="100" dataDxfId="22"/>
+  </tableColumns>
+  <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
+</table>
+</file>
+
+<file path=xl/tables/table9.xml><?xml version="1.0" encoding="utf-8"?>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="9" xr:uid="{ED109B1C-F705-4CDA-A157-70FDD3DCBAEA}" name="Table9" displayName="Table9" ref="A1:F11" totalsRowShown="0" dataDxfId="14" tableBorderDxfId="20">
+  <autoFilter ref="A1:F11" xr:uid="{ED109B1C-F705-4CDA-A157-70FDD3DCBAEA}"/>
+  <tableColumns count="6">
+    <tableColumn id="1" xr3:uid="{12913906-ADCA-4787-A8C5-E858FAB3B40E}" name="20"/>
+    <tableColumn id="2" xr3:uid="{69CC8094-647F-474C-9AD5-926E2ECFC91E}" name="25" dataDxfId="19"/>
+    <tableColumn id="3" xr3:uid="{3F4FE94F-C203-4AFB-B01C-6FE570AA28E3}" name="40" dataDxfId="18"/>
+    <tableColumn id="4" xr3:uid="{071C23C4-2565-4CA3-810F-355E14305750}" name="50" dataDxfId="17"/>
+    <tableColumn id="5" xr3:uid="{ADA5EBD9-87B7-4CF4-931A-D9BCD8E63C54}" name="75" dataDxfId="16"/>
+    <tableColumn id="6" xr3:uid="{564FB2FC-4EF7-4C12-A20D-F11ADCE26D64}" name="100" dataDxfId="15"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -7200,6 +8069,472 @@
 </worksheet>
 </file>
 
+<file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{02B0D750-DDAA-4327-9449-D0F93D1C9F9A}">
+  <dimension ref="A1:F11"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetData>
+    <row r="1" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A1" t="s">
+        <v>277</v>
+      </c>
+      <c r="B1" t="s">
+        <v>278</v>
+      </c>
+      <c r="C1" t="s">
+        <v>279</v>
+      </c>
+      <c r="D1" t="s">
+        <v>280</v>
+      </c>
+      <c r="E1" t="s">
+        <v>281</v>
+      </c>
+      <c r="F1" t="s">
+        <v>282</v>
+      </c>
+    </row>
+    <row r="2" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A2" s="7">
+        <v>9.0659749999758704E-2</v>
+      </c>
+      <c r="B2" s="7">
+        <v>0.123557750000145</v>
+      </c>
+      <c r="C2" s="7">
+        <v>0.82291654199980202</v>
+      </c>
+      <c r="D2" s="7">
+        <v>2.7484046260005899</v>
+      </c>
+      <c r="E2" s="7">
+        <v>25.6964639699999</v>
+      </c>
+      <c r="F2" s="7">
+        <v>3.32769850099975</v>
+      </c>
+    </row>
+    <row r="3" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A3" s="8">
+        <v>5.8049999999639099E-2</v>
+      </c>
+      <c r="B3" s="8">
+        <v>0.174720875000275</v>
+      </c>
+      <c r="C3" s="8">
+        <v>0.88722950099963704</v>
+      </c>
+      <c r="D3" s="8">
+        <v>4.3689845439994297</v>
+      </c>
+      <c r="E3" s="8">
+        <v>25.0604030530003</v>
+      </c>
+      <c r="F3" s="8">
+        <v>43.969725020000602</v>
+      </c>
+    </row>
+    <row r="4" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A4" s="7">
+        <v>5.3727833000266401E-2</v>
+      </c>
+      <c r="B4" s="7">
+        <v>0.12626474999979101</v>
+      </c>
+      <c r="C4" s="7">
+        <v>0.81283458399957398</v>
+      </c>
+      <c r="D4" s="7">
+        <v>4.7785656269998</v>
+      </c>
+      <c r="E4" s="7">
+        <v>13.9307466729997</v>
+      </c>
+      <c r="F4" s="7">
+        <v>105.602236048999</v>
+      </c>
+    </row>
+    <row r="5" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A5" s="8">
+        <v>5.4628792000585201E-2</v>
+      </c>
+      <c r="B5" s="8">
+        <v>0.103825333000713</v>
+      </c>
+      <c r="C5" s="8">
+        <v>0.79964345899952605</v>
+      </c>
+      <c r="D5" s="8">
+        <v>1.92413308400045</v>
+      </c>
+      <c r="E5" s="8">
+        <v>18.090029300000399</v>
+      </c>
+      <c r="F5" s="8">
+        <v>69.539149072999805</v>
+      </c>
+    </row>
+    <row r="6" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A6" s="7">
+        <v>6.7796667000038696E-2</v>
+      </c>
+      <c r="B6" s="7">
+        <v>0.10428475000026</v>
+      </c>
+      <c r="C6" s="7">
+        <v>1.5188525009998499</v>
+      </c>
+      <c r="D6" s="7">
+        <v>2.4920137510007399</v>
+      </c>
+      <c r="E6" s="7">
+        <v>18.773501841999799</v>
+      </c>
+      <c r="F6" s="7">
+        <v>95.267819126000106</v>
+      </c>
+    </row>
+    <row r="7" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A7" s="8">
+        <v>5.9643624999807798E-2</v>
+      </c>
+      <c r="B7" s="8">
+        <v>0.10405258399987299</v>
+      </c>
+      <c r="C7" s="8">
+        <v>0.87141316699944504</v>
+      </c>
+      <c r="D7" s="8">
+        <v>2.0492544589997101</v>
+      </c>
+      <c r="E7" s="8">
+        <v>13.0287071299999</v>
+      </c>
+      <c r="F7" s="8">
+        <v>44.019741561999503</v>
+      </c>
+    </row>
+    <row r="8" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A8" s="7">
+        <v>7.3612582999885406E-2</v>
+      </c>
+      <c r="B8" s="7">
+        <v>0.11870591700062499</v>
+      </c>
+      <c r="C8" s="7">
+        <v>0.97011229200052096</v>
+      </c>
+      <c r="D8" s="7">
+        <v>3.97414858499996</v>
+      </c>
+      <c r="E8" s="7">
+        <v>3.9797428349993398</v>
+      </c>
+      <c r="F8" s="7">
+        <v>55.732546899999697</v>
+      </c>
+    </row>
+    <row r="9" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A9" s="8">
+        <v>7.1703583000271395E-2</v>
+      </c>
+      <c r="B9" s="8">
+        <v>9.3496290999610196E-2</v>
+      </c>
+      <c r="C9" s="8">
+        <v>1.67325000100026</v>
+      </c>
+      <c r="D9" s="8">
+        <v>2.47690783400048</v>
+      </c>
+      <c r="E9" s="8">
+        <v>6.0642318359996299</v>
+      </c>
+      <c r="F9" s="8">
+        <v>28.185838387999802</v>
+      </c>
+    </row>
+    <row r="10" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A10" s="7">
+        <v>7.0189584000218005E-2</v>
+      </c>
+      <c r="B10" s="7">
+        <v>0.14683254099963899</v>
+      </c>
+      <c r="C10" s="7">
+        <v>1.0260740840003499</v>
+      </c>
+      <c r="D10" s="7">
+        <v>2.8002696270004801</v>
+      </c>
+      <c r="E10" s="7">
+        <v>6.8716945449996203</v>
+      </c>
+      <c r="F10" s="7">
+        <v>77.706257493999999</v>
+      </c>
+    </row>
+    <row r="11" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A11" s="11">
+        <v>4.1546958999788303E-2</v>
+      </c>
+      <c r="B11" s="12">
+        <v>5.12649590000364E-2</v>
+      </c>
+      <c r="C11" s="12">
+        <v>1.18243399999937</v>
+      </c>
+      <c r="D11" s="12">
+        <v>3.28088875100002</v>
+      </c>
+      <c r="E11" s="12">
+        <v>30.645577221999702</v>
+      </c>
+      <c r="F11" s="12">
+        <v>33.318394347999799</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <tableParts count="1">
+    <tablePart r:id="rId1"/>
+  </tableParts>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{9E31298D-DB3B-404D-8EF4-AD7B0DACAA41}">
+  <dimension ref="A1:F11"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetData>
+    <row r="1" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A1" t="s">
+        <v>277</v>
+      </c>
+      <c r="B1" t="s">
+        <v>278</v>
+      </c>
+      <c r="C1" t="s">
+        <v>279</v>
+      </c>
+      <c r="D1" t="s">
+        <v>280</v>
+      </c>
+      <c r="E1" t="s">
+        <v>281</v>
+      </c>
+      <c r="F1" t="s">
+        <v>282</v>
+      </c>
+    </row>
+    <row r="2" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A2" s="9">
+        <v>0.16066162499919301</v>
+      </c>
+      <c r="B2" s="9">
+        <v>0.19009912499950499</v>
+      </c>
+      <c r="C2" s="9">
+        <v>2.42598616599934</v>
+      </c>
+      <c r="D2" s="9">
+        <v>18.026117092000199</v>
+      </c>
+      <c r="E2" s="9">
+        <v>159.59676973800001</v>
+      </c>
+      <c r="F2" s="9">
+        <v>87.265396372999007</v>
+      </c>
+    </row>
+    <row r="3" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A3" s="10">
+        <v>8.8539541999125504E-2</v>
+      </c>
+      <c r="B3" s="10">
+        <v>0.24558804200023501</v>
+      </c>
+      <c r="C3" s="10">
+        <v>4.9841860440001202</v>
+      </c>
+      <c r="D3" s="10">
+        <v>15.811426299999701</v>
+      </c>
+      <c r="E3" s="10">
+        <v>177.60294691299899</v>
+      </c>
+      <c r="F3" s="10">
+        <v>156.993464821</v>
+      </c>
+    </row>
+    <row r="4" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A4" s="9">
+        <v>9.3913083999723299E-2</v>
+      </c>
+      <c r="B4" s="9">
+        <v>0.18059608299972699</v>
+      </c>
+      <c r="C4" s="9">
+        <v>1.8357979590000399</v>
+      </c>
+      <c r="D4" s="9">
+        <v>13.6218335060002</v>
+      </c>
+      <c r="E4" s="9">
+        <v>85.405975870999995</v>
+      </c>
+      <c r="F4" s="9">
+        <v>899.17824857400001</v>
+      </c>
+    </row>
+    <row r="5" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A5" s="10">
+        <v>8.8027249999868204E-2</v>
+      </c>
+      <c r="B5" s="10">
+        <v>0.26194841599954</v>
+      </c>
+      <c r="C5" s="10">
+        <v>3.6631602939996801</v>
+      </c>
+      <c r="D5" s="10">
+        <v>4.00780341800054</v>
+      </c>
+      <c r="E5" s="10">
+        <v>96.128000085000096</v>
+      </c>
+      <c r="F5" s="10">
+        <v>681.20098185200004</v>
+      </c>
+    </row>
+    <row r="6" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A6" s="9">
+        <v>0.15493399999832</v>
+      </c>
+      <c r="B6" s="9">
+        <v>0.194003292000161</v>
+      </c>
+      <c r="C6" s="9">
+        <v>4.3989879189994099</v>
+      </c>
+      <c r="D6" s="9">
+        <v>18.430154466999699</v>
+      </c>
+      <c r="E6" s="9">
+        <v>70.043700572999995</v>
+      </c>
+      <c r="F6" s="9">
+        <v>331.37683652599998</v>
+      </c>
+    </row>
+    <row r="7" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A7" s="10">
+        <v>0.24887812500128301</v>
+      </c>
+      <c r="B7" s="10">
+        <v>0.30845104099989801</v>
+      </c>
+      <c r="C7" s="10">
+        <v>3.1248001260000802</v>
+      </c>
+      <c r="D7" s="10">
+        <v>6.93431383700044</v>
+      </c>
+      <c r="E7" s="10">
+        <v>56.528150317999398</v>
+      </c>
+      <c r="F7" s="10">
+        <v>549.05003112499901</v>
+      </c>
+    </row>
+    <row r="8" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A8" s="9">
+        <v>0.113710666999395</v>
+      </c>
+      <c r="B8" s="9">
+        <v>0.29773333400044</v>
+      </c>
+      <c r="C8" s="9">
+        <v>8.9091196710005498</v>
+      </c>
+      <c r="D8" s="9">
+        <v>14.789426590000399</v>
+      </c>
+      <c r="E8" s="9">
+        <v>21.245699134999899</v>
+      </c>
+      <c r="F8" s="9">
+        <v>367.492057958001</v>
+      </c>
+    </row>
+    <row r="9" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A9" s="10">
+        <v>0.18527125100081299</v>
+      </c>
+      <c r="B9" s="10">
+        <v>0.16896749999978</v>
+      </c>
+      <c r="C9" s="10">
+        <v>8.0786281290002009</v>
+      </c>
+      <c r="D9" s="10">
+        <v>13.3802078809994</v>
+      </c>
+      <c r="E9" s="10">
+        <v>40.264259976998801</v>
+      </c>
+      <c r="F9" s="10">
+        <v>203.371497341999</v>
+      </c>
+    </row>
+    <row r="10" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A10" s="9">
+        <v>0.102808667001227</v>
+      </c>
+      <c r="B10" s="9">
+        <v>0.29684416700001698</v>
+      </c>
+      <c r="C10" s="9">
+        <v>2.1229899179998002</v>
+      </c>
+      <c r="D10" s="9">
+        <v>7.0354148360002</v>
+      </c>
+      <c r="E10" s="9">
+        <v>37.626907600000699</v>
+      </c>
+      <c r="F10" s="9">
+        <v>430.75752302799901</v>
+      </c>
+    </row>
+    <row r="11" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A11" s="13">
+        <v>9.9966666999534895E-2</v>
+      </c>
+      <c r="B11" s="14">
+        <v>0.151434417000018</v>
+      </c>
+      <c r="C11" s="14">
+        <v>3.3875301259995401</v>
+      </c>
+      <c r="D11" s="14">
+        <v>20.098683342000101</v>
+      </c>
+      <c r="E11" s="14">
+        <v>236.93741298399999</v>
+      </c>
+      <c r="F11" s="14">
+        <v>142.233111815001</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <tableParts count="1">
+    <tablePart r:id="rId1"/>
+  </tableParts>
+</worksheet>
+</file>
+
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{57B4A7D9-29A4-43B1-B1C6-F7F43184D58B}">
   <dimension ref="A1:J18"/>
@@ -12412,4 +13747,1707 @@
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F969AA13-E93D-4FB3-98B1-0A08B32216AC}">
+  <dimension ref="A1:F61"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="3" max="3" width="18" bestFit="1" customWidth="1"/>
+    <col min="4" max="6" width="16.85546875" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" t="s">
+        <v>13</v>
+      </c>
+      <c r="C1" t="s">
+        <v>10</v>
+      </c>
+      <c r="D1" t="s">
+        <v>201</v>
+      </c>
+      <c r="E1" t="s">
+        <v>219</v>
+      </c>
+      <c r="F1" t="s">
+        <v>234</v>
+      </c>
+    </row>
+    <row r="2" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A2">
+        <v>52</v>
+      </c>
+      <c r="B2">
+        <v>20</v>
+      </c>
+      <c r="C2">
+        <v>3.7240982055664002E-3</v>
+      </c>
+      <c r="D2">
+        <v>5.78074999998534E-2</v>
+      </c>
+      <c r="E2">
+        <v>9.0659749999758704E-2</v>
+      </c>
+      <c r="F2">
+        <v>0.16066162499919301</v>
+      </c>
+    </row>
+    <row r="3" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A3">
+        <v>53</v>
+      </c>
+      <c r="B3">
+        <v>20</v>
+      </c>
+      <c r="C3">
+        <v>3.6454200744628902E-3</v>
+      </c>
+      <c r="D3">
+        <v>3.9888125000288703E-2</v>
+      </c>
+      <c r="E3">
+        <v>5.8049999999639099E-2</v>
+      </c>
+      <c r="F3">
+        <v>8.8539541999125504E-2</v>
+      </c>
+    </row>
+    <row r="4" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A4">
+        <v>60</v>
+      </c>
+      <c r="B4">
+        <v>20</v>
+      </c>
+      <c r="C4">
+        <v>3.8189888000488199E-3</v>
+      </c>
+      <c r="D4">
+        <v>2.8228874999967901E-2</v>
+      </c>
+      <c r="E4">
+        <v>5.3727833000266401E-2</v>
+      </c>
+      <c r="F4">
+        <v>9.3913083999723299E-2</v>
+      </c>
+    </row>
+    <row r="5" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A5">
+        <v>54</v>
+      </c>
+      <c r="B5">
+        <v>20</v>
+      </c>
+      <c r="C5">
+        <v>3.5321712493896402E-3</v>
+      </c>
+      <c r="D5">
+        <v>2.8433916999802002E-2</v>
+      </c>
+      <c r="E5">
+        <v>5.4628792000585201E-2</v>
+      </c>
+      <c r="F5">
+        <v>8.8027249999868204E-2</v>
+      </c>
+    </row>
+    <row r="6" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A6">
+        <v>58</v>
+      </c>
+      <c r="B6">
+        <v>20</v>
+      </c>
+      <c r="C6">
+        <v>3.5631656646728498E-3</v>
+      </c>
+      <c r="D6">
+        <v>4.4324792000224898E-2</v>
+      </c>
+      <c r="E6">
+        <v>6.7796667000038696E-2</v>
+      </c>
+      <c r="F6">
+        <v>0.15493399999832</v>
+      </c>
+    </row>
+    <row r="7" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A7">
+        <v>57</v>
+      </c>
+      <c r="B7">
+        <v>20</v>
+      </c>
+      <c r="C7">
+        <v>3.5440921783447201E-3</v>
+      </c>
+      <c r="D7">
+        <v>4.8121415999958103E-2</v>
+      </c>
+      <c r="E7">
+        <v>5.9643624999807798E-2</v>
+      </c>
+      <c r="F7">
+        <v>0.24887812500128301</v>
+      </c>
+    </row>
+    <row r="8" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A8">
+        <v>56</v>
+      </c>
+      <c r="B8">
+        <v>20</v>
+      </c>
+      <c r="C8">
+        <v>3.4809112548828099E-3</v>
+      </c>
+      <c r="D8">
+        <v>5.5611165999834997E-2</v>
+      </c>
+      <c r="E8">
+        <v>7.3612582999885406E-2</v>
+      </c>
+      <c r="F8">
+        <v>0.113710666999395</v>
+      </c>
+    </row>
+    <row r="9" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A9">
+        <v>59</v>
+      </c>
+      <c r="B9">
+        <v>20</v>
+      </c>
+      <c r="C9">
+        <v>3.4942626953125E-3</v>
+      </c>
+      <c r="D9">
+        <v>1.50465840001743E-2</v>
+      </c>
+      <c r="E9">
+        <v>7.1703583000271395E-2</v>
+      </c>
+      <c r="F9">
+        <v>0.18527125100081299</v>
+      </c>
+    </row>
+    <row r="10" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A10">
+        <v>51</v>
+      </c>
+      <c r="B10">
+        <v>20</v>
+      </c>
+      <c r="C10">
+        <v>4.2831897735595703E-3</v>
+      </c>
+      <c r="D10">
+        <v>4.4080166999719901E-2</v>
+      </c>
+      <c r="E10">
+        <v>7.0189584000218005E-2</v>
+      </c>
+      <c r="F10">
+        <v>0.102808667001227</v>
+      </c>
+    </row>
+    <row r="11" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A11" s="5">
+        <v>55</v>
+      </c>
+      <c r="B11" s="5">
+        <v>20</v>
+      </c>
+      <c r="C11" s="5">
+        <v>3.5791397094726502E-3</v>
+      </c>
+      <c r="D11" s="5">
+        <v>6.6444000000046799E-2</v>
+      </c>
+      <c r="E11" s="5">
+        <v>4.1546958999788303E-2</v>
+      </c>
+      <c r="F11" s="5">
+        <v>9.9966666999534895E-2</v>
+      </c>
+    </row>
+    <row r="12" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A12">
+        <v>10</v>
+      </c>
+      <c r="B12">
+        <v>25</v>
+      </c>
+      <c r="C12">
+        <v>4.1575431823730399E-3</v>
+      </c>
+      <c r="D12">
+        <v>6.4846166999814103E-2</v>
+      </c>
+      <c r="E12">
+        <v>0.123557750000145</v>
+      </c>
+      <c r="F12">
+        <v>0.19009912499950499</v>
+      </c>
+    </row>
+    <row r="13" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A13">
+        <v>2</v>
+      </c>
+      <c r="B13">
+        <v>25</v>
+      </c>
+      <c r="C13">
+        <v>4.5094490051269497E-3</v>
+      </c>
+      <c r="D13">
+        <v>5.3255167000315802E-2</v>
+      </c>
+      <c r="E13">
+        <v>0.174720875000275</v>
+      </c>
+      <c r="F13">
+        <v>0.24558804200023501</v>
+      </c>
+    </row>
+    <row r="14" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A14">
+        <v>5</v>
+      </c>
+      <c r="B14">
+        <v>25</v>
+      </c>
+      <c r="C14">
+        <v>4.1453838348388602E-3</v>
+      </c>
+      <c r="D14">
+        <v>2.0007292000173E-2</v>
+      </c>
+      <c r="E14">
+        <v>0.12626474999979101</v>
+      </c>
+      <c r="F14">
+        <v>0.18059608299972699</v>
+      </c>
+    </row>
+    <row r="15" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A15">
+        <v>3</v>
+      </c>
+      <c r="B15">
+        <v>25</v>
+      </c>
+      <c r="C15">
+        <v>4.02426719665527E-3</v>
+      </c>
+      <c r="D15">
+        <v>2.7863165999860901E-2</v>
+      </c>
+      <c r="E15">
+        <v>0.103825333000713</v>
+      </c>
+      <c r="F15">
+        <v>0.26194841599954</v>
+      </c>
+    </row>
+    <row r="16" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A16">
+        <v>6</v>
+      </c>
+      <c r="B16">
+        <v>25</v>
+      </c>
+      <c r="C16">
+        <v>4.6305656433105399E-3</v>
+      </c>
+      <c r="D16">
+        <v>4.92233330000999E-2</v>
+      </c>
+      <c r="E16">
+        <v>0.10428475000026</v>
+      </c>
+      <c r="F16">
+        <v>0.194003292000161</v>
+      </c>
+    </row>
+    <row r="17" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A17">
+        <v>8</v>
+      </c>
+      <c r="B17">
+        <v>25</v>
+      </c>
+      <c r="C17">
+        <v>4.3210983276367101E-3</v>
+      </c>
+      <c r="D17">
+        <v>5.1922249999734001E-2</v>
+      </c>
+      <c r="E17">
+        <v>0.10405258399987299</v>
+      </c>
+      <c r="F17">
+        <v>0.30845104099989801</v>
+      </c>
+    </row>
+    <row r="18" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A18">
+        <v>7</v>
+      </c>
+      <c r="B18">
+        <v>25</v>
+      </c>
+      <c r="C18">
+        <v>4.2986869812011701E-3</v>
+      </c>
+      <c r="D18">
+        <v>5.5771708000065701E-2</v>
+      </c>
+      <c r="E18">
+        <v>0.11870591700062499</v>
+      </c>
+      <c r="F18">
+        <v>0.29773333400044</v>
+      </c>
+    </row>
+    <row r="19" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A19">
+        <v>9</v>
+      </c>
+      <c r="B19">
+        <v>25</v>
+      </c>
+      <c r="C19">
+        <v>4.4243335723876901E-3</v>
+      </c>
+      <c r="D19">
+        <v>5.66445829999793E-2</v>
+      </c>
+      <c r="E19">
+        <v>9.3496290999610196E-2</v>
+      </c>
+      <c r="F19">
+        <v>0.16896749999978</v>
+      </c>
+    </row>
+    <row r="20" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A20">
+        <v>1</v>
+      </c>
+      <c r="B20">
+        <v>25</v>
+      </c>
+      <c r="C20">
+        <v>1.48313045501708E-2</v>
+      </c>
+      <c r="D20">
+        <v>6.3491874999726805E-2</v>
+      </c>
+      <c r="E20">
+        <v>0.14683254099963899</v>
+      </c>
+      <c r="F20">
+        <v>0.29684416700001698</v>
+      </c>
+    </row>
+    <row r="21" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A21">
+        <v>4</v>
+      </c>
+      <c r="B21">
+        <v>25</v>
+      </c>
+      <c r="C21">
+        <v>4.1053295135498004E-3</v>
+      </c>
+      <c r="D21">
+        <v>5.1364457999625301E-2</v>
+      </c>
+      <c r="E21">
+        <v>5.12649590000364E-2</v>
+      </c>
+      <c r="F21">
+        <v>0.151434417000018</v>
+      </c>
+    </row>
+    <row r="22" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A22">
+        <v>11</v>
+      </c>
+      <c r="B22">
+        <v>40</v>
+      </c>
+      <c r="C22">
+        <v>5.05590438842773E-3</v>
+      </c>
+      <c r="D22">
+        <v>0.168602750000445</v>
+      </c>
+      <c r="E22">
+        <v>0.82291654199980202</v>
+      </c>
+      <c r="F22">
+        <v>2.42598616599934</v>
+      </c>
+    </row>
+    <row r="23" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A23">
+        <v>14</v>
+      </c>
+      <c r="B23">
+        <v>40</v>
+      </c>
+      <c r="C23">
+        <v>5.0327777862548802E-3</v>
+      </c>
+      <c r="D23">
+        <v>7.4470166000082799E-2</v>
+      </c>
+      <c r="E23">
+        <v>0.88722950099963704</v>
+      </c>
+      <c r="F23">
+        <v>4.9841860440001202</v>
+      </c>
+    </row>
+    <row r="24" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A24">
+        <v>15</v>
+      </c>
+      <c r="B24">
+        <v>40</v>
+      </c>
+      <c r="C24">
+        <v>4.9045085906982396E-3</v>
+      </c>
+      <c r="D24">
+        <v>8.8303416000144297E-2</v>
+      </c>
+      <c r="E24">
+        <v>0.81283458399957398</v>
+      </c>
+      <c r="F24">
+        <v>1.8357979590000399</v>
+      </c>
+    </row>
+    <row r="25" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A25">
+        <v>19</v>
+      </c>
+      <c r="B25">
+        <v>40</v>
+      </c>
+      <c r="C25">
+        <v>4.7674179077148403E-3</v>
+      </c>
+      <c r="D25">
+        <v>9.3740249999882494E-2</v>
+      </c>
+      <c r="E25">
+        <v>0.79964345899952605</v>
+      </c>
+      <c r="F25">
+        <v>3.6631602939996801</v>
+      </c>
+    </row>
+    <row r="26" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A26">
+        <v>12</v>
+      </c>
+      <c r="B26">
+        <v>40</v>
+      </c>
+      <c r="C26">
+        <v>4.7380924224853498E-3</v>
+      </c>
+      <c r="D26">
+        <v>0.103318750000198</v>
+      </c>
+      <c r="E26">
+        <v>1.5188525009998499</v>
+      </c>
+      <c r="F26">
+        <v>4.3989879189994099</v>
+      </c>
+    </row>
+    <row r="27" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A27">
+        <v>18</v>
+      </c>
+      <c r="B27">
+        <v>40</v>
+      </c>
+      <c r="C27">
+        <v>5.3415298461914002E-3</v>
+      </c>
+      <c r="D27">
+        <v>0.11625504199992</v>
+      </c>
+      <c r="E27">
+        <v>0.87141316699944504</v>
+      </c>
+      <c r="F27">
+        <v>3.1248001260000802</v>
+      </c>
+    </row>
+    <row r="28" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A28">
+        <v>13</v>
+      </c>
+      <c r="B28">
+        <v>40</v>
+      </c>
+      <c r="C28">
+        <v>4.8034191131591797E-3</v>
+      </c>
+      <c r="D28">
+        <v>0.13974787500001101</v>
+      </c>
+      <c r="E28">
+        <v>0.97011229200052096</v>
+      </c>
+      <c r="F28">
+        <v>8.9091196710005498</v>
+      </c>
+    </row>
+    <row r="29" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A29">
+        <v>20</v>
+      </c>
+      <c r="B29">
+        <v>40</v>
+      </c>
+      <c r="C29">
+        <v>4.8246383666992101E-3</v>
+      </c>
+      <c r="D29">
+        <v>0.202652332999605</v>
+      </c>
+      <c r="E29">
+        <v>1.67325000100026</v>
+      </c>
+      <c r="F29">
+        <v>8.0786281290002009</v>
+      </c>
+    </row>
+    <row r="30" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A30">
+        <v>17</v>
+      </c>
+      <c r="B30">
+        <v>40</v>
+      </c>
+      <c r="C30">
+        <v>4.7316551208495998E-3</v>
+      </c>
+      <c r="D30">
+        <v>0.116587292000076</v>
+      </c>
+      <c r="E30">
+        <v>1.0260740840003499</v>
+      </c>
+      <c r="F30">
+        <v>2.1229899179998002</v>
+      </c>
+    </row>
+    <row r="31" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A31">
+        <v>16</v>
+      </c>
+      <c r="B31">
+        <v>40</v>
+      </c>
+      <c r="C31">
+        <v>4.8835277557373004E-3</v>
+      </c>
+      <c r="D31">
+        <v>0.20691229200019701</v>
+      </c>
+      <c r="E31">
+        <v>1.18243399999937</v>
+      </c>
+      <c r="F31">
+        <v>3.3875301259995401</v>
+      </c>
+    </row>
+    <row r="32" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A32">
+        <v>24</v>
+      </c>
+      <c r="B32">
+        <v>50</v>
+      </c>
+      <c r="C32">
+        <v>6.07061386108398E-3</v>
+      </c>
+      <c r="D32">
+        <v>0.38118024999994299</v>
+      </c>
+      <c r="E32">
+        <v>2.7484046260005899</v>
+      </c>
+      <c r="F32">
+        <v>18.026117092000199</v>
+      </c>
+    </row>
+    <row r="33" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A33">
+        <v>26</v>
+      </c>
+      <c r="B33">
+        <v>50</v>
+      </c>
+      <c r="C33">
+        <v>5.63573837280273E-3</v>
+      </c>
+      <c r="D33">
+        <v>0.28343674999996399</v>
+      </c>
+      <c r="E33">
+        <v>4.3689845439994297</v>
+      </c>
+      <c r="F33">
+        <v>15.811426299999701</v>
+      </c>
+    </row>
+    <row r="34" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A34">
+        <v>22</v>
+      </c>
+      <c r="B34">
+        <v>50</v>
+      </c>
+      <c r="C34">
+        <v>5.5255889892578099E-3</v>
+      </c>
+      <c r="D34">
+        <v>0.40008525000030198</v>
+      </c>
+      <c r="E34">
+        <v>4.7785656269998</v>
+      </c>
+      <c r="F34">
+        <v>13.6218335060002</v>
+      </c>
+    </row>
+    <row r="35" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A35">
+        <v>27</v>
+      </c>
+      <c r="B35">
+        <v>50</v>
+      </c>
+      <c r="C35">
+        <v>5.7203769683837804E-3</v>
+      </c>
+      <c r="D35">
+        <v>0.15869841599987899</v>
+      </c>
+      <c r="E35">
+        <v>1.92413308400045</v>
+      </c>
+      <c r="F35">
+        <v>4.00780341800054</v>
+      </c>
+    </row>
+    <row r="36" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A36">
+        <v>21</v>
+      </c>
+      <c r="B36">
+        <v>50</v>
+      </c>
+      <c r="C36">
+        <v>5.3641796112060504E-3</v>
+      </c>
+      <c r="D36">
+        <v>0.165316750000329</v>
+      </c>
+      <c r="E36">
+        <v>2.4920137510007399</v>
+      </c>
+      <c r="F36">
+        <v>18.430154466999699</v>
+      </c>
+    </row>
+    <row r="37" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A37">
+        <v>30</v>
+      </c>
+      <c r="B37">
+        <v>50</v>
+      </c>
+      <c r="C37">
+        <v>6.0241222381591797E-3</v>
+      </c>
+      <c r="D37">
+        <v>0.20384345899992601</v>
+      </c>
+      <c r="E37">
+        <v>2.0492544589997101</v>
+      </c>
+      <c r="F37">
+        <v>6.93431383700044</v>
+      </c>
+    </row>
+    <row r="38" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A38">
+        <v>29</v>
+      </c>
+      <c r="B38">
+        <v>50</v>
+      </c>
+      <c r="C38">
+        <v>5.5742263793945304E-3</v>
+      </c>
+      <c r="D38">
+        <v>0.30268154199984498</v>
+      </c>
+      <c r="E38">
+        <v>3.97414858499996</v>
+      </c>
+      <c r="F38">
+        <v>14.789426590000399</v>
+      </c>
+    </row>
+    <row r="39" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A39">
+        <v>25</v>
+      </c>
+      <c r="B39">
+        <v>50</v>
+      </c>
+      <c r="C39">
+        <v>5.7797431945800703E-3</v>
+      </c>
+      <c r="D39">
+        <v>0.193798458999935</v>
+      </c>
+      <c r="E39">
+        <v>2.47690783400048</v>
+      </c>
+      <c r="F39">
+        <v>13.3802078809994</v>
+      </c>
+    </row>
+    <row r="40" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A40">
+        <v>28</v>
+      </c>
+      <c r="B40">
+        <v>50</v>
+      </c>
+      <c r="C40">
+        <v>5.7938098907470703E-3</v>
+      </c>
+      <c r="D40">
+        <v>0.25469179199990299</v>
+      </c>
+      <c r="E40">
+        <v>2.8002696270004801</v>
+      </c>
+      <c r="F40">
+        <v>7.0354148360002</v>
+      </c>
+    </row>
+    <row r="41" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A41">
+        <v>23</v>
+      </c>
+      <c r="B41">
+        <v>50</v>
+      </c>
+      <c r="C41">
+        <v>5.6612491607665998E-3</v>
+      </c>
+      <c r="D41">
+        <v>0.33562787599976202</v>
+      </c>
+      <c r="E41">
+        <v>3.28088875100002</v>
+      </c>
+      <c r="F41">
+        <v>20.098683342000101</v>
+      </c>
+    </row>
+    <row r="42" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A42">
+        <v>37</v>
+      </c>
+      <c r="B42">
+        <v>75</v>
+      </c>
+      <c r="C42">
+        <v>6.9537162780761701E-3</v>
+      </c>
+      <c r="D42">
+        <v>1.9745873339997999</v>
+      </c>
+      <c r="E42">
+        <v>25.6964639699999</v>
+      </c>
+      <c r="F42">
+        <v>159.59676973800001</v>
+      </c>
+    </row>
+    <row r="43" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A43">
+        <v>33</v>
+      </c>
+      <c r="B43">
+        <v>75</v>
+      </c>
+      <c r="C43">
+        <v>7.4980258941650304E-3</v>
+      </c>
+      <c r="D43">
+        <v>0.82913062499983403</v>
+      </c>
+      <c r="E43">
+        <v>25.0604030530003</v>
+      </c>
+      <c r="F43">
+        <v>177.60294691299899</v>
+      </c>
+    </row>
+    <row r="44" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A44">
+        <v>34</v>
+      </c>
+      <c r="B44">
+        <v>75</v>
+      </c>
+      <c r="C44">
+        <v>7.43985176086425E-3</v>
+      </c>
+      <c r="D44">
+        <v>0.43395962500016999</v>
+      </c>
+      <c r="E44">
+        <v>13.9307466729997</v>
+      </c>
+      <c r="F44">
+        <v>85.405975870999995</v>
+      </c>
+    </row>
+    <row r="45" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A45">
+        <v>32</v>
+      </c>
+      <c r="B45">
+        <v>75</v>
+      </c>
+      <c r="C45">
+        <v>7.1249008178710903E-3</v>
+      </c>
+      <c r="D45">
+        <v>0.52399945800016201</v>
+      </c>
+      <c r="E45">
+        <v>18.090029300000399</v>
+      </c>
+      <c r="F45">
+        <v>96.128000085000096</v>
+      </c>
+    </row>
+    <row r="46" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A46">
+        <v>35</v>
+      </c>
+      <c r="B46">
+        <v>75</v>
+      </c>
+      <c r="C46">
+        <v>7.4191093444824201E-3</v>
+      </c>
+      <c r="D46">
+        <v>0.73774899999989396</v>
+      </c>
+      <c r="E46">
+        <v>18.773501841999799</v>
+      </c>
+      <c r="F46">
+        <v>70.043700572999995</v>
+      </c>
+    </row>
+    <row r="47" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A47">
+        <v>31</v>
+      </c>
+      <c r="B47">
+        <v>75</v>
+      </c>
+      <c r="C47">
+        <v>7.2510242462158203E-3</v>
+      </c>
+      <c r="D47">
+        <v>0.85136941800010302</v>
+      </c>
+      <c r="E47">
+        <v>13.0287071299999</v>
+      </c>
+      <c r="F47">
+        <v>56.528150317999398</v>
+      </c>
+    </row>
+    <row r="48" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A48">
+        <v>36</v>
+      </c>
+      <c r="B48">
+        <v>75</v>
+      </c>
+      <c r="C48">
+        <v>7.6315402984619097E-3</v>
+      </c>
+      <c r="D48">
+        <v>0.48733279199996099</v>
+      </c>
+      <c r="E48">
+        <v>3.9797428349993398</v>
+      </c>
+      <c r="F48">
+        <v>21.245699134999899</v>
+      </c>
+    </row>
+    <row r="49" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A49">
+        <v>40</v>
+      </c>
+      <c r="B49">
+        <v>75</v>
+      </c>
+      <c r="C49">
+        <v>7.6365470886230399E-3</v>
+      </c>
+      <c r="D49">
+        <v>1.2455521669999099</v>
+      </c>
+      <c r="E49">
+        <v>6.0642318359996299</v>
+      </c>
+      <c r="F49">
+        <v>40.264259976998801</v>
+      </c>
+    </row>
+    <row r="50" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A50">
+        <v>39</v>
+      </c>
+      <c r="B50">
+        <v>75</v>
+      </c>
+      <c r="C50">
+        <v>7.1530342102050703E-3</v>
+      </c>
+      <c r="D50">
+        <v>0.74755229199990902</v>
+      </c>
+      <c r="E50">
+        <v>6.8716945449996203</v>
+      </c>
+      <c r="F50">
+        <v>37.626907600000699</v>
+      </c>
+    </row>
+    <row r="51" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A51">
+        <v>38</v>
+      </c>
+      <c r="B51">
+        <v>75</v>
+      </c>
+      <c r="C51">
+        <v>6.7458152770995998E-3</v>
+      </c>
+      <c r="D51">
+        <v>7.0090071280001203</v>
+      </c>
+      <c r="E51">
+        <v>30.645577221999702</v>
+      </c>
+      <c r="F51">
+        <v>236.93741298399999</v>
+      </c>
+    </row>
+    <row r="52" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A52">
+        <v>48</v>
+      </c>
+      <c r="B52">
+        <v>100</v>
+      </c>
+      <c r="C52">
+        <v>9.0699195861816406E-3</v>
+      </c>
+      <c r="D52">
+        <v>1.23514304200034</v>
+      </c>
+      <c r="E52">
+        <v>3.32769850099975</v>
+      </c>
+      <c r="F52">
+        <v>87.265396372999007</v>
+      </c>
+    </row>
+    <row r="53" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A53">
+        <v>47</v>
+      </c>
+      <c r="B53">
+        <v>100</v>
+      </c>
+      <c r="C53">
+        <v>9.4974040985107405E-3</v>
+      </c>
+      <c r="D53">
+        <v>1.2422580009997499</v>
+      </c>
+      <c r="E53">
+        <v>43.969725020000602</v>
+      </c>
+      <c r="F53">
+        <v>156.993464821</v>
+      </c>
+    </row>
+    <row r="54" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A54">
+        <v>41</v>
+      </c>
+      <c r="B54">
+        <v>100</v>
+      </c>
+      <c r="C54">
+        <v>9.1185569763183594E-3</v>
+      </c>
+      <c r="D54">
+        <v>4.4783545440000099</v>
+      </c>
+      <c r="E54">
+        <v>105.602236048999</v>
+      </c>
+      <c r="F54">
+        <v>899.17824857400001</v>
+      </c>
+    </row>
+    <row r="55" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A55">
+        <v>44</v>
+      </c>
+      <c r="B55">
+        <v>100</v>
+      </c>
+      <c r="C55">
+        <v>8.6023807525634696E-3</v>
+      </c>
+      <c r="D55">
+        <v>1.67711304199974</v>
+      </c>
+      <c r="E55">
+        <v>69.539149072999805</v>
+      </c>
+      <c r="F55">
+        <v>681.20098185200004</v>
+      </c>
+    </row>
+    <row r="56" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A56">
+        <v>43</v>
+      </c>
+      <c r="B56">
+        <v>100</v>
+      </c>
+      <c r="C56">
+        <v>8.9905261993408203E-3</v>
+      </c>
+      <c r="D56">
+        <v>2.6676563349997102</v>
+      </c>
+      <c r="E56">
+        <v>95.267819126000106</v>
+      </c>
+      <c r="F56">
+        <v>331.37683652599998</v>
+      </c>
+    </row>
+    <row r="57" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A57">
+        <v>49</v>
+      </c>
+      <c r="B57">
+        <v>100</v>
+      </c>
+      <c r="C57">
+        <v>8.8615417480468698E-3</v>
+      </c>
+      <c r="D57">
+        <v>2.9854539190000602</v>
+      </c>
+      <c r="E57">
+        <v>44.019741561999503</v>
+      </c>
+      <c r="F57">
+        <v>549.05003112499901</v>
+      </c>
+    </row>
+    <row r="58" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A58">
+        <v>50</v>
+      </c>
+      <c r="B58">
+        <v>100</v>
+      </c>
+      <c r="C58">
+        <v>8.8996887207031198E-3</v>
+      </c>
+      <c r="D58">
+        <v>1.1968654590000301</v>
+      </c>
+      <c r="E58">
+        <v>55.732546899999697</v>
+      </c>
+      <c r="F58">
+        <v>367.492057958001</v>
+      </c>
+    </row>
+    <row r="59" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A59">
+        <v>42</v>
+      </c>
+      <c r="B59">
+        <v>100</v>
+      </c>
+      <c r="C59">
+        <v>8.72802734375E-3</v>
+      </c>
+      <c r="D59">
+        <v>1.51752133400032</v>
+      </c>
+      <c r="E59">
+        <v>28.185838387999802</v>
+      </c>
+      <c r="F59">
+        <v>203.371497341999</v>
+      </c>
+    </row>
+    <row r="60" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A60">
+        <v>45</v>
+      </c>
+      <c r="B60">
+        <v>100</v>
+      </c>
+      <c r="C60">
+        <v>8.9101791381835903E-3</v>
+      </c>
+      <c r="D60">
+        <v>2.6582356270000602</v>
+      </c>
+      <c r="E60">
+        <v>77.706257493999999</v>
+      </c>
+      <c r="F60">
+        <v>430.75752302799901</v>
+      </c>
+    </row>
+    <row r="61" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A61">
+        <v>46</v>
+      </c>
+      <c r="B61">
+        <v>100</v>
+      </c>
+      <c r="C61">
+        <v>8.9771747589111293E-3</v>
+      </c>
+      <c r="D61">
+        <v>1.88445083500027</v>
+      </c>
+      <c r="E61">
+        <v>33.318394347999799</v>
+      </c>
+      <c r="F61">
+        <v>142.233111815001</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <tableParts count="1">
+    <tablePart r:id="rId1"/>
+  </tableParts>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{4DFDB532-E6A4-45BD-AE21-4D7D5D9046BE}">
+  <dimension ref="A1:F11"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetData>
+    <row r="1" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A1" t="s">
+        <v>277</v>
+      </c>
+      <c r="B1" t="s">
+        <v>278</v>
+      </c>
+      <c r="C1" t="s">
+        <v>279</v>
+      </c>
+      <c r="D1" t="s">
+        <v>280</v>
+      </c>
+      <c r="E1" t="s">
+        <v>281</v>
+      </c>
+      <c r="F1" t="s">
+        <v>282</v>
+      </c>
+    </row>
+    <row r="2" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A2" s="7">
+        <v>3.7240982055664002E-3</v>
+      </c>
+      <c r="B2" s="7">
+        <v>4.1575431823730399E-3</v>
+      </c>
+      <c r="C2" s="7">
+        <v>5.05590438842773E-3</v>
+      </c>
+      <c r="D2" s="7">
+        <v>6.07061386108398E-3</v>
+      </c>
+      <c r="E2" s="7">
+        <v>6.9537162780761701E-3</v>
+      </c>
+      <c r="F2" s="7">
+        <v>9.0699195861816406E-3</v>
+      </c>
+    </row>
+    <row r="3" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A3" s="8">
+        <v>3.6454200744628902E-3</v>
+      </c>
+      <c r="B3" s="8">
+        <v>4.5094490051269497E-3</v>
+      </c>
+      <c r="C3" s="8">
+        <v>5.0327777862548802E-3</v>
+      </c>
+      <c r="D3" s="8">
+        <v>5.63573837280273E-3</v>
+      </c>
+      <c r="E3" s="8">
+        <v>7.4980258941650304E-3</v>
+      </c>
+      <c r="F3" s="8">
+        <v>9.4974040985107405E-3</v>
+      </c>
+    </row>
+    <row r="4" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A4" s="7">
+        <v>3.8189888000488199E-3</v>
+      </c>
+      <c r="B4" s="7">
+        <v>4.1453838348388602E-3</v>
+      </c>
+      <c r="C4" s="7">
+        <v>4.9045085906982396E-3</v>
+      </c>
+      <c r="D4" s="7">
+        <v>5.5255889892578099E-3</v>
+      </c>
+      <c r="E4" s="7">
+        <v>7.43985176086425E-3</v>
+      </c>
+      <c r="F4" s="7">
+        <v>9.1185569763183594E-3</v>
+      </c>
+    </row>
+    <row r="5" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A5" s="8">
+        <v>3.5321712493896402E-3</v>
+      </c>
+      <c r="B5" s="8">
+        <v>4.02426719665527E-3</v>
+      </c>
+      <c r="C5" s="8">
+        <v>4.7674179077148403E-3</v>
+      </c>
+      <c r="D5" s="8">
+        <v>5.7203769683837804E-3</v>
+      </c>
+      <c r="E5" s="8">
+        <v>7.1249008178710903E-3</v>
+      </c>
+      <c r="F5" s="8">
+        <v>8.6023807525634696E-3</v>
+      </c>
+    </row>
+    <row r="6" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A6" s="7">
+        <v>3.5631656646728498E-3</v>
+      </c>
+      <c r="B6" s="7">
+        <v>4.6305656433105399E-3</v>
+      </c>
+      <c r="C6" s="7">
+        <v>4.7380924224853498E-3</v>
+      </c>
+      <c r="D6" s="7">
+        <v>5.3641796112060504E-3</v>
+      </c>
+      <c r="E6" s="7">
+        <v>7.4191093444824201E-3</v>
+      </c>
+      <c r="F6" s="7">
+        <v>8.9905261993408203E-3</v>
+      </c>
+    </row>
+    <row r="7" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A7" s="8">
+        <v>3.5440921783447201E-3</v>
+      </c>
+      <c r="B7" s="8">
+        <v>4.3210983276367101E-3</v>
+      </c>
+      <c r="C7" s="8">
+        <v>5.3415298461914002E-3</v>
+      </c>
+      <c r="D7" s="8">
+        <v>6.0241222381591797E-3</v>
+      </c>
+      <c r="E7" s="8">
+        <v>7.2510242462158203E-3</v>
+      </c>
+      <c r="F7" s="8">
+        <v>8.8615417480468698E-3</v>
+      </c>
+    </row>
+    <row r="8" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A8" s="7">
+        <v>3.4809112548828099E-3</v>
+      </c>
+      <c r="B8" s="7">
+        <v>4.2986869812011701E-3</v>
+      </c>
+      <c r="C8" s="7">
+        <v>4.8034191131591797E-3</v>
+      </c>
+      <c r="D8" s="7">
+        <v>5.5742263793945304E-3</v>
+      </c>
+      <c r="E8" s="7">
+        <v>7.6315402984619097E-3</v>
+      </c>
+      <c r="F8" s="7">
+        <v>8.8996887207031198E-3</v>
+      </c>
+    </row>
+    <row r="9" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A9" s="8">
+        <v>3.4942626953125E-3</v>
+      </c>
+      <c r="B9" s="8">
+        <v>4.4243335723876901E-3</v>
+      </c>
+      <c r="C9" s="8">
+        <v>4.8246383666992101E-3</v>
+      </c>
+      <c r="D9" s="8">
+        <v>5.7797431945800703E-3</v>
+      </c>
+      <c r="E9" s="8">
+        <v>7.6365470886230399E-3</v>
+      </c>
+      <c r="F9" s="8">
+        <v>8.72802734375E-3</v>
+      </c>
+    </row>
+    <row r="10" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A10" s="7">
+        <v>4.2831897735595703E-3</v>
+      </c>
+      <c r="B10" s="7">
+        <v>1.48313045501708E-2</v>
+      </c>
+      <c r="C10" s="7">
+        <v>4.7316551208495998E-3</v>
+      </c>
+      <c r="D10" s="7">
+        <v>5.7938098907470703E-3</v>
+      </c>
+      <c r="E10" s="7">
+        <v>7.1530342102050703E-3</v>
+      </c>
+      <c r="F10" s="7">
+        <v>8.9101791381835903E-3</v>
+      </c>
+    </row>
+    <row r="11" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A11" s="11">
+        <v>3.5791397094726502E-3</v>
+      </c>
+      <c r="B11" s="12">
+        <v>4.1053295135498004E-3</v>
+      </c>
+      <c r="C11" s="12">
+        <v>4.8835277557373004E-3</v>
+      </c>
+      <c r="D11" s="12">
+        <v>5.6612491607665998E-3</v>
+      </c>
+      <c r="E11" s="12">
+        <v>6.7458152770995998E-3</v>
+      </c>
+      <c r="F11" s="12">
+        <v>8.9771747589111293E-3</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <tableParts count="1">
+    <tablePart r:id="rId1"/>
+  </tableParts>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C25D4473-F029-42A7-89A5-6EE5A2C2DB67}">
+  <dimension ref="A1:F11"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetData>
+    <row r="1" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A1" t="s">
+        <v>277</v>
+      </c>
+      <c r="B1" t="s">
+        <v>278</v>
+      </c>
+      <c r="C1" t="s">
+        <v>279</v>
+      </c>
+      <c r="D1" t="s">
+        <v>280</v>
+      </c>
+      <c r="E1" t="s">
+        <v>281</v>
+      </c>
+      <c r="F1" t="s">
+        <v>282</v>
+      </c>
+    </row>
+    <row r="2" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A2" s="7">
+        <v>5.78074999998534E-2</v>
+      </c>
+      <c r="B2" s="7">
+        <v>6.4846166999814103E-2</v>
+      </c>
+      <c r="C2" s="7">
+        <v>0.168602750000445</v>
+      </c>
+      <c r="D2" s="7">
+        <v>0.38118024999994299</v>
+      </c>
+      <c r="E2" s="7">
+        <v>1.9745873339997999</v>
+      </c>
+      <c r="F2" s="7">
+        <v>1.23514304200034</v>
+      </c>
+    </row>
+    <row r="3" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A3" s="8">
+        <v>3.9888125000288703E-2</v>
+      </c>
+      <c r="B3" s="8">
+        <v>5.3255167000315802E-2</v>
+      </c>
+      <c r="C3" s="8">
+        <v>7.4470166000082799E-2</v>
+      </c>
+      <c r="D3" s="8">
+        <v>0.28343674999996399</v>
+      </c>
+      <c r="E3" s="8">
+        <v>0.82913062499983403</v>
+      </c>
+      <c r="F3" s="8">
+        <v>1.2422580009997499</v>
+      </c>
+    </row>
+    <row r="4" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A4" s="7">
+        <v>2.8228874999967901E-2</v>
+      </c>
+      <c r="B4" s="7">
+        <v>2.0007292000173E-2</v>
+      </c>
+      <c r="C4" s="7">
+        <v>8.8303416000144297E-2</v>
+      </c>
+      <c r="D4" s="7">
+        <v>0.40008525000030198</v>
+      </c>
+      <c r="E4" s="7">
+        <v>0.43395962500016999</v>
+      </c>
+      <c r="F4" s="7">
+        <v>4.4783545440000099</v>
+      </c>
+    </row>
+    <row r="5" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A5" s="8">
+        <v>2.8433916999802002E-2</v>
+      </c>
+      <c r="B5" s="8">
+        <v>2.7863165999860901E-2</v>
+      </c>
+      <c r="C5" s="8">
+        <v>9.3740249999882494E-2</v>
+      </c>
+      <c r="D5" s="8">
+        <v>0.15869841599987899</v>
+      </c>
+      <c r="E5" s="8">
+        <v>0.52399945800016201</v>
+      </c>
+      <c r="F5" s="8">
+        <v>1.67711304199974</v>
+      </c>
+    </row>
+    <row r="6" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A6" s="7">
+        <v>4.4324792000224898E-2</v>
+      </c>
+      <c r="B6" s="7">
+        <v>4.92233330000999E-2</v>
+      </c>
+      <c r="C6" s="7">
+        <v>0.103318750000198</v>
+      </c>
+      <c r="D6" s="7">
+        <v>0.165316750000329</v>
+      </c>
+      <c r="E6" s="7">
+        <v>0.73774899999989396</v>
+      </c>
+      <c r="F6" s="7">
+        <v>2.6676563349997102</v>
+      </c>
+    </row>
+    <row r="7" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A7" s="8">
+        <v>4.8121415999958103E-2</v>
+      </c>
+      <c r="B7" s="8">
+        <v>5.1922249999734001E-2</v>
+      </c>
+      <c r="C7" s="8">
+        <v>0.11625504199992</v>
+      </c>
+      <c r="D7" s="8">
+        <v>0.20384345899992601</v>
+      </c>
+      <c r="E7" s="8">
+        <v>0.85136941800010302</v>
+      </c>
+      <c r="F7" s="8">
+        <v>2.9854539190000602</v>
+      </c>
+    </row>
+    <row r="8" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A8" s="7">
+        <v>5.5611165999834997E-2</v>
+      </c>
+      <c r="B8" s="7">
+        <v>5.5771708000065701E-2</v>
+      </c>
+      <c r="C8" s="7">
+        <v>0.13974787500001101</v>
+      </c>
+      <c r="D8" s="7">
+        <v>0.30268154199984498</v>
+      </c>
+      <c r="E8" s="7">
+        <v>0.48733279199996099</v>
+      </c>
+      <c r="F8" s="7">
+        <v>1.1968654590000301</v>
+      </c>
+    </row>
+    <row r="9" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A9" s="8">
+        <v>1.50465840001743E-2</v>
+      </c>
+      <c r="B9" s="8">
+        <v>5.66445829999793E-2</v>
+      </c>
+      <c r="C9" s="8">
+        <v>0.202652332999605</v>
+      </c>
+      <c r="D9" s="8">
+        <v>0.193798458999935</v>
+      </c>
+      <c r="E9" s="8">
+        <v>1.2455521669999099</v>
+      </c>
+      <c r="F9" s="8">
+        <v>1.51752133400032</v>
+      </c>
+    </row>
+    <row r="10" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A10" s="7">
+        <v>4.4080166999719901E-2</v>
+      </c>
+      <c r="B10" s="7">
+        <v>6.3491874999726805E-2</v>
+      </c>
+      <c r="C10" s="7">
+        <v>0.116587292000076</v>
+      </c>
+      <c r="D10" s="7">
+        <v>0.25469179199990299</v>
+      </c>
+      <c r="E10" s="7">
+        <v>0.74755229199990902</v>
+      </c>
+      <c r="F10" s="7">
+        <v>2.6582356270000602</v>
+      </c>
+    </row>
+    <row r="11" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A11" s="11">
+        <v>6.6444000000046799E-2</v>
+      </c>
+      <c r="B11" s="12">
+        <v>5.1364457999625301E-2</v>
+      </c>
+      <c r="C11" s="12">
+        <v>0.20691229200019701</v>
+      </c>
+      <c r="D11" s="12">
+        <v>0.33562787599976202</v>
+      </c>
+      <c r="E11" s="12">
+        <v>7.0090071280001203</v>
+      </c>
+      <c r="F11" s="12">
+        <v>1.88445083500027</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <tableParts count="1">
+    <tablePart r:id="rId1"/>
+  </tableParts>
+</worksheet>
 </file>
</xml_diff>